<commit_message>
Refactored Tabs logic in app.py, Added Hyderabad data and Hyderabad tab. Added some schema checks in schema_utils.py
</commit_message>
<xml_diff>
--- a/data/Vapi/Spinning.xlsx
+++ b/data/Vapi/Spinning.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Nikhitha\OneDrive\Desktop\Manning_AUM\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\099901939\WLL\production\manning\data\Vapi\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A27A5A94-B1FD-49F2-9F70-8465DE6A863E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="12460" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Spinning" sheetId="1" r:id="rId1"/>
@@ -19,7 +18,7 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Spinning!$A$1:$T$117</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -35,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="953" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="873" uniqueCount="286">
   <si>
     <t>Location</t>
   </si>
@@ -826,18 +825,6 @@
     <t>RFID Tag Application &amp; Unloading &amp; Laydown</t>
   </si>
   <si>
-    <t>ROUNDUP((((SUM(T2:T18)/36)+(T19/36))*3),0)</t>
-  </si>
-  <si>
-    <t>ROUND(ROUNDUP(T19,0)/16,0)*2</t>
-  </si>
-  <si>
-    <t>ROUND(+SUM(N2:N18)/6,0)*3</t>
-  </si>
-  <si>
-    <t>ROUNDUP(+SUM(N2:N18)/4,0)*3</t>
-  </si>
-  <si>
     <t>BLOW ROOM OPERATOR</t>
   </si>
   <si>
@@ -893,12 +880,24 @@
   </si>
   <si>
     <t>Dept_Machine_Name</t>
+  </si>
+  <si>
+    <t>ROUNDUP((((SUM(TFO!T2:T18)/36)+(TFO!T19/36))*3),0)</t>
+  </si>
+  <si>
+    <t>ROUND(ROUNDUP(TFO!T19,0)/16,0)*2</t>
+  </si>
+  <si>
+    <t>ROUND(+SUM(TFO!N2:N18)/6,0)*3</t>
+  </si>
+  <si>
+    <t>ROUNDUP(+SUM(TFO!N2:N18)/4,0)*3</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1001,7 +1000,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1020,7 +1018,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1039,7 +1036,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1058,7 +1054,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1077,7 +1072,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1096,7 +1090,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1115,7 +1108,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1134,7 +1126,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1153,7 +1144,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1172,7 +1162,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1191,7 +1180,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1210,7 +1198,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1229,7 +1216,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1248,7 +1234,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1267,7 +1252,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1286,7 +1270,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1305,7 +1288,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1324,7 +1306,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1349,7 +1330,6 @@
         <sz val="11"/>
         <color rgb="FF000000"/>
         <name val="Calibri"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </font>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -1368,72 +1348,72 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F622A60C-E8BF-4683-BFA8-DC9CDCD99FD8}" name="Table1" displayName="Table1" ref="A1:T117" totalsRowShown="0" dataDxfId="30">
-  <autoFilter ref="A1:T117" xr:uid="{F622A60C-E8BF-4683-BFA8-DC9CDCD99FD8}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Table1" displayName="Table1" ref="A1:T117" totalsRowShown="0" dataDxfId="30">
+  <autoFilter ref="A1:T117"/>
   <tableColumns count="20">
-    <tableColumn id="1" xr3:uid="{85A1F019-9DB7-48AC-AF2B-F0C9FBE637DA}" name="Location" dataDxfId="29"/>
-    <tableColumn id="2" xr3:uid="{545588E2-5E30-4A62-AB93-1DBC57F6BCF8}" name="Business" dataDxfId="28"/>
-    <tableColumn id="3" xr3:uid="{44C3C497-13A6-40FF-AABF-EC930E13E039}" name="Section" dataDxfId="27"/>
-    <tableColumn id="4" xr3:uid="{ED8F8366-2CFD-45B1-B1C2-AA92F55B23F6}" name="Sr_No" dataDxfId="26"/>
-    <tableColumn id="5" xr3:uid="{3C440E90-56BF-4BC4-ACD0-A73E98969A14}" name="Dept_Machine_Name" dataDxfId="25"/>
-    <tableColumn id="6" xr3:uid="{EADE3DD8-7C1C-4874-8032-AD8F2F81A125}" name="Designation" dataDxfId="24"/>
-    <tableColumn id="7" xr3:uid="{292F7B89-A9FA-4B1D-8581-9D4596E679FF}" name="Machine_Count" dataDxfId="23"/>
-    <tableColumn id="9" xr3:uid="{090D3B71-C4CF-432F-B817-104F30316591}" name="Workload" dataDxfId="22"/>
-    <tableColumn id="10" xr3:uid="{9EDB9484-B177-478C-9BA3-4C1AE3030F95}" name="Formulas" dataDxfId="21"/>
-    <tableColumn id="11" xr3:uid="{3A1186F6-9294-4AEC-A543-A07372ADEF4D}" name="BE_Scientific_Manpower" dataDxfId="20"/>
-    <tableColumn id="20" xr3:uid="{071CCBE0-65D5-467E-AFCC-8949549E1BB6}" name="Operator_Type" dataDxfId="19"/>
-    <tableColumn id="8" xr3:uid="{F5544431-B0F5-4C79-B5EB-61614939F4B5}" name="Contractors" dataDxfId="18"/>
-    <tableColumn id="19" xr3:uid="{15BE4AF0-E211-4DE0-800A-0EDB9C705B37}" name="Company_Associate" dataDxfId="17"/>
-    <tableColumn id="12" xr3:uid="{47E45710-4EB9-4699-B8AD-09AC38DE8C54}" name="BE_Final_Manpower" dataDxfId="16"/>
-    <tableColumn id="13" xr3:uid="{38203A5B-662C-436E-A752-C238B552EF03}" name="General_Shift" dataDxfId="15"/>
-    <tableColumn id="14" xr3:uid="{3D149A8F-3122-4C7E-B50D-02B6DF1691E0}" name="Shift_A" dataDxfId="14"/>
-    <tableColumn id="15" xr3:uid="{0AFA7034-EEDB-4D14-A601-C01016D3A7D5}" name="Shift_B" dataDxfId="13"/>
-    <tableColumn id="16" xr3:uid="{64D43A66-597F-4C18-84E0-E76FCB0F95CC}" name="Shift_C" dataDxfId="12"/>
-    <tableColumn id="17" xr3:uid="{554EDC51-4B6D-44FF-BB2C-DA6797B32110}" name="Reliever" dataDxfId="11"/>
-    <tableColumn id="18" xr3:uid="{FF4E975E-F83C-4D1D-8950-072C414D6E58}" name="Remarks" dataDxfId="10"/>
+    <tableColumn id="1" name="Location" dataDxfId="29"/>
+    <tableColumn id="2" name="Business" dataDxfId="28"/>
+    <tableColumn id="3" name="Section" dataDxfId="27"/>
+    <tableColumn id="4" name="Sr_No" dataDxfId="26"/>
+    <tableColumn id="5" name="Dept_Machine_Name" dataDxfId="25"/>
+    <tableColumn id="6" name="Designation" dataDxfId="24"/>
+    <tableColumn id="7" name="Machine_Count" dataDxfId="23"/>
+    <tableColumn id="9" name="Workload" dataDxfId="22"/>
+    <tableColumn id="10" name="Formulas" dataDxfId="21"/>
+    <tableColumn id="11" name="BE_Scientific_Manpower" dataDxfId="20"/>
+    <tableColumn id="20" name="Operator_Type" dataDxfId="19"/>
+    <tableColumn id="8" name="Contractors" dataDxfId="18"/>
+    <tableColumn id="19" name="Company_Associate" dataDxfId="17"/>
+    <tableColumn id="12" name="BE_Final_Manpower" dataDxfId="16"/>
+    <tableColumn id="13" name="General_Shift" dataDxfId="15"/>
+    <tableColumn id="14" name="Shift_A" dataDxfId="14"/>
+    <tableColumn id="15" name="Shift_B" dataDxfId="13"/>
+    <tableColumn id="16" name="Shift_C" dataDxfId="12"/>
+    <tableColumn id="17" name="Reliever" dataDxfId="11"/>
+    <tableColumn id="18" name="Remarks" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{1A41DC54-EC66-4CAB-9BBF-6CB0CD4E37DB}" name="Table2" displayName="Table2" ref="A1:X19" totalsRowShown="0">
-  <autoFilter ref="A1:X19" xr:uid="{1A41DC54-EC66-4CAB-9BBF-6CB0CD4E37DB}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="Table2" displayName="Table2" ref="A1:X19" totalsRowShown="0">
+  <autoFilter ref="A1:X19"/>
   <tableColumns count="24">
-    <tableColumn id="1" xr3:uid="{1DCD2645-4593-4E7F-A866-0402A47C5590}" name="Count"/>
-    <tableColumn id="2" xr3:uid="{ECB8C04A-41DB-4ACF-BDD5-35648226FD4D}" name="Customer"/>
-    <tableColumn id="3" xr3:uid="{7FB2A76E-99F2-4234-BB76-1E7500BC87DA}" name="Count2"/>
-    <tableColumn id="4" xr3:uid="{9FCFBAC9-9818-49B9-A38A-0BBF74E1AF08}" name="Speed"/>
-    <tableColumn id="5" xr3:uid="{CF7EB0B9-C0A6-469A-A583-452612604A93}" name="TPI"/>
-    <tableColumn id="6" xr3:uid="{FBED24A1-3DB2-4325-BDD9-BCEFD8DBE7E0}" name="Utilization"/>
-    <tableColumn id="7" xr3:uid="{00039784-93D4-4F03-94F0-3D9165F3F7B5}" name="Efficiency"/>
-    <tableColumn id="8" xr3:uid="{1C0BCECE-7E25-429A-A07A-493E05A1B64D}" name="Formula_Production per Drum/ day "/>
-    <tableColumn id="9" xr3:uid="{A45DFE32-A98D-4B00-AA84-34B653FFF353}" name="Production per Drum/ day ">
+    <tableColumn id="1" name="Count"/>
+    <tableColumn id="2" name="Customer"/>
+    <tableColumn id="3" name="Count2"/>
+    <tableColumn id="4" name="Speed"/>
+    <tableColumn id="5" name="TPI"/>
+    <tableColumn id="6" name="Utilization"/>
+    <tableColumn id="7" name="Efficiency"/>
+    <tableColumn id="8" name="Formula_Production per Drum/ day "/>
+    <tableColumn id="9" name="Production per Drum/ day ">
       <calculatedColumnFormula>((D2*60*8*G2*2)/(E2*36*840*C2*2.202))*3</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="23" xr3:uid="{C69696E1-455D-46A2-A34D-ED761D3A9E4E}" name="formula_Production Required / Month Kgs "/>
-    <tableColumn id="10" xr3:uid="{0CE5E939-1885-4A81-9F54-45019D6AF9ED}" name="Production Required / Month Kgs ">
+    <tableColumn id="23" name="formula_Production Required / Month Kgs "/>
+    <tableColumn id="10" name="Production Required / Month Kgs ">
       <calculatedColumnFormula>L2*30</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{2D9BB7FC-414D-44A7-BA33-064AB74254EC}" name="Production Required / day  Kgs "/>
-    <tableColumn id="24" xr3:uid="{837B0BC7-A2DA-48D8-B881-2E9004073921}" name="formul_No. of Drums Required"/>
-    <tableColumn id="12" xr3:uid="{E2B4A990-ABE7-4090-BE7B-CE105F913FDC}" name="No. of Drums Required">
+    <tableColumn id="11" name="Production Required / day  Kgs "/>
+    <tableColumn id="24" name="formul_No. of Drums Required"/>
+    <tableColumn id="12" name="No. of Drums Required">
       <calculatedColumnFormula>L2/I2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{7C882653-B2FB-4460-945F-BEC827034FAE}" name="formula_No. of TFO Required/ shift "/>
-    <tableColumn id="14" xr3:uid="{74DD064C-08DB-4132-A242-1290AD15CDB8}" name="No. of TFO Required/ shift " dataDxfId="9" totalsRowDxfId="8"/>
-    <tableColumn id="15" xr3:uid="{65F3003E-C476-4D6D-BE1A-6488E17CDB9D}" name="mpm"/>
-    <tableColumn id="16" xr3:uid="{6E9D763E-DE2C-4A86-B1EA-5287AC19467B}" name="Eff" dataDxfId="7" totalsRowDxfId="6"/>
-    <tableColumn id="17" xr3:uid="{4C4EE216-BFC8-45EA-BA92-DA7C3E734438}" name="Formula_kgs/drum/day " dataDxfId="5" totalsRowDxfId="4"/>
-    <tableColumn id="18" xr3:uid="{00170897-62B8-4C84-AE04-5EAE44ABC362}" name="kgs/drum/day ">
+    <tableColumn id="13" name="formula_No. of TFO Required/ shift "/>
+    <tableColumn id="14" name="No. of TFO Required/ shift " dataDxfId="9" totalsRowDxfId="8"/>
+    <tableColumn id="15" name="mpm"/>
+    <tableColumn id="16" name="Eff" dataDxfId="7" totalsRowDxfId="6"/>
+    <tableColumn id="17" name="Formula_kgs/drum/day " dataDxfId="5" totalsRowDxfId="4"/>
+    <tableColumn id="18" name="kgs/drum/day ">
       <calculatedColumnFormula>Q2*R2*8*60*1.09/(C2*840*2.202)*3</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="19" xr3:uid="{2DD7DB04-94B4-4773-9E4C-D99D0E582A8C}" name="formula_No. of Drums"/>
-    <tableColumn id="20" xr3:uid="{B964DFB3-EA94-419A-8A86-F1F5917ADCA3}" name="No. of Drums " dataDxfId="3" totalsRowDxfId="2">
+    <tableColumn id="19" name="formula_No. of Drums"/>
+    <tableColumn id="20" name="No. of Drums " dataDxfId="3" totalsRowDxfId="2">
       <calculatedColumnFormula>L2/T2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="21" xr3:uid="{ACA15BF8-B0A7-481E-A7F2-D7E94E5D9CB0}" name="formula_no. of machines" dataDxfId="1" totalsRowDxfId="0"/>
-    <tableColumn id="22" xr3:uid="{0459E32F-2AB6-434A-9439-F5F08B7C6254}" name="no. of machines">
+    <tableColumn id="21" name="formula_no. of machines" dataDxfId="1" totalsRowDxfId="0"/>
+    <tableColumn id="22" name="no. of machines">
       <calculatedColumnFormula>V2/72</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -1725,28 +1705,28 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:T117"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.109375" customWidth="1"/>
-    <col min="2" max="2" width="13.33203125" customWidth="1"/>
-    <col min="3" max="3" width="20.109375" customWidth="1"/>
-    <col min="4" max="4" width="10.109375" customWidth="1"/>
-    <col min="5" max="5" width="46.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="44.44140625" customWidth="1"/>
-    <col min="7" max="7" width="20.77734375" customWidth="1"/>
-    <col min="8" max="8" width="48.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.08984375" customWidth="1"/>
+    <col min="2" max="2" width="13.36328125" customWidth="1"/>
+    <col min="3" max="3" width="20.08984375" customWidth="1"/>
+    <col min="4" max="4" width="10.08984375" customWidth="1"/>
+    <col min="5" max="5" width="46.81640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="44.453125" customWidth="1"/>
+    <col min="7" max="7" width="20.81640625" customWidth="1"/>
+    <col min="8" max="8" width="48.453125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="40" bestFit="1" customWidth="1"/>
-    <col min="10" max="13" width="31.5546875" customWidth="1"/>
-    <col min="14" max="14" width="26.21875" customWidth="1"/>
-    <col min="15" max="15" width="18.77734375" customWidth="1"/>
-    <col min="16" max="18" width="11.5546875" customWidth="1"/>
-    <col min="19" max="19" width="12.33203125" customWidth="1"/>
-    <col min="20" max="20" width="38.6640625" customWidth="1"/>
+    <col min="10" max="13" width="31.54296875" customWidth="1"/>
+    <col min="14" max="14" width="26.1796875" customWidth="1"/>
+    <col min="15" max="15" width="18.81640625" customWidth="1"/>
+    <col min="16" max="18" width="11.54296875" customWidth="1"/>
+    <col min="19" max="19" width="12.36328125" customWidth="1"/>
+    <col min="20" max="20" width="38.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1760,7 +1740,7 @@
         <v>2</v>
       </c>
       <c r="E1" t="s">
-        <v>285</v>
+        <v>281</v>
       </c>
       <c r="F1" t="s">
         <v>3</v>
@@ -1775,19 +1755,19 @@
         <v>45</v>
       </c>
       <c r="J1" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="K1" t="s">
-        <v>284</v>
+        <v>280</v>
       </c>
       <c r="L1" t="s">
         <v>42</v>
       </c>
       <c r="M1" t="s">
-        <v>283</v>
+        <v>279</v>
       </c>
       <c r="N1" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="O1" t="s">
         <v>5</v>
@@ -1808,7 +1788,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -1825,7 +1805,7 @@
         <v>14</v>
       </c>
       <c r="F2" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="G2">
         <v>8</v>
@@ -1861,7 +1841,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -1911,7 +1891,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -1961,7 +1941,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>11</v>
       </c>
@@ -2011,7 +1991,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>11</v>
       </c>
@@ -2061,7 +2041,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>11</v>
       </c>
@@ -2111,7 +2091,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>11</v>
       </c>
@@ -2161,7 +2141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>11</v>
       </c>
@@ -2211,7 +2191,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>11</v>
       </c>
@@ -2261,7 +2241,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>11</v>
       </c>
@@ -2314,7 +2294,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -2364,7 +2344,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -2411,7 +2391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>11</v>
       </c>
@@ -2458,7 +2438,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>11</v>
       </c>
@@ -2505,7 +2485,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>11</v>
       </c>
@@ -2528,7 +2508,7 @@
         <v>43</v>
       </c>
       <c r="I16" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="J16">
         <v>0</v>
@@ -2555,7 +2535,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>11</v>
       </c>
@@ -2605,7 +2585,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>11</v>
       </c>
@@ -2655,7 +2635,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>11</v>
       </c>
@@ -2705,7 +2685,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A20" t="s">
         <v>11</v>
       </c>
@@ -2755,7 +2735,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A21" t="s">
         <v>11</v>
       </c>
@@ -2802,7 +2782,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A22" t="s">
         <v>11</v>
       </c>
@@ -2852,7 +2832,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A23" t="s">
         <v>11</v>
       </c>
@@ -2902,7 +2882,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A24" t="s">
         <v>11</v>
       </c>
@@ -2952,7 +2932,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A25" t="s">
         <v>11</v>
       </c>
@@ -3002,7 +2982,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A26" t="s">
         <v>11</v>
       </c>
@@ -3052,7 +3032,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A27" t="s">
         <v>11</v>
       </c>
@@ -3099,7 +3079,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A28" t="s">
         <v>11</v>
       </c>
@@ -3149,7 +3129,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A29" t="s">
         <v>11</v>
       </c>
@@ -3196,7 +3176,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A30" t="s">
         <v>11</v>
       </c>
@@ -3243,7 +3223,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="31" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A31" t="s">
         <v>11</v>
       </c>
@@ -3290,7 +3270,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="32" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A32" t="s">
         <v>11</v>
       </c>
@@ -3337,7 +3317,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A33" t="s">
         <v>11</v>
       </c>
@@ -3384,7 +3364,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A34" t="s">
         <v>11</v>
       </c>
@@ -3431,7 +3411,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A35" t="s">
         <v>11</v>
       </c>
@@ -3475,7 +3455,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A36" t="s">
         <v>11</v>
       </c>
@@ -3522,7 +3502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A37" t="s">
         <v>11</v>
       </c>
@@ -3542,7 +3522,7 @@
         <v>6</v>
       </c>
       <c r="H37" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="I37" t="s">
         <v>105</v>
@@ -3569,7 +3549,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A38" t="s">
         <v>11</v>
       </c>
@@ -3613,7 +3593,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A39" t="s">
         <v>11</v>
       </c>
@@ -3657,7 +3637,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A40" t="s">
         <v>11</v>
       </c>
@@ -3704,7 +3684,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A41" t="s">
         <v>11</v>
       </c>
@@ -3724,7 +3704,7 @@
         <v>107</v>
       </c>
       <c r="I41" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="J41">
         <v>1</v>
@@ -3751,7 +3731,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A42" t="s">
         <v>11</v>
       </c>
@@ -3798,7 +3778,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A43" t="s">
         <v>11</v>
       </c>
@@ -3845,7 +3825,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A44" t="s">
         <v>11</v>
       </c>
@@ -3892,7 +3872,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A45" t="s">
         <v>11</v>
       </c>
@@ -3939,7 +3919,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A46" t="s">
         <v>11</v>
       </c>
@@ -3989,7 +3969,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="47" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A47" t="s">
         <v>11</v>
       </c>
@@ -4039,7 +4019,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="48" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A48" t="s">
         <v>11</v>
       </c>
@@ -4089,7 +4069,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A49" t="s">
         <v>11</v>
       </c>
@@ -4133,7 +4113,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A50" t="s">
         <v>11</v>
       </c>
@@ -4153,7 +4133,7 @@
         <v>121</v>
       </c>
       <c r="I50" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="J50">
         <v>1</v>
@@ -4177,7 +4157,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A51" t="s">
         <v>11</v>
       </c>
@@ -4225,7 +4205,7 @@
       </c>
       <c r="T51" s="4"/>
     </row>
-    <row r="52" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A52" s="1" t="s">
         <v>11</v>
       </c>
@@ -4273,7 +4253,7 @@
       </c>
       <c r="T52" s="4"/>
     </row>
-    <row r="53" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A53" s="1" t="s">
         <v>11</v>
       </c>
@@ -4321,7 +4301,7 @@
       </c>
       <c r="T53" s="4"/>
     </row>
-    <row r="54" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A54" s="1" t="s">
         <v>11</v>
       </c>
@@ -4369,7 +4349,7 @@
       </c>
       <c r="T54" s="1"/>
     </row>
-    <row r="55" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A55" s="1" t="s">
         <v>11</v>
       </c>
@@ -4419,7 +4399,7 @@
       </c>
       <c r="T55" s="1"/>
     </row>
-    <row r="56" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A56" s="1" t="s">
         <v>11</v>
       </c>
@@ -4469,7 +4449,7 @@
       </c>
       <c r="T56" s="1"/>
     </row>
-    <row r="57" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A57" s="1" t="s">
         <v>11</v>
       </c>
@@ -4519,7 +4499,7 @@
       </c>
       <c r="T57" s="1"/>
     </row>
-    <row r="58" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A58" s="1" t="s">
         <v>11</v>
       </c>
@@ -4571,7 +4551,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="59" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A59" s="1" t="s">
         <v>11</v>
       </c>
@@ -4621,7 +4601,7 @@
       </c>
       <c r="T59" s="1"/>
     </row>
-    <row r="60" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A60" s="1" t="s">
         <v>11</v>
       </c>
@@ -4671,7 +4651,7 @@
       </c>
       <c r="T60" s="1"/>
     </row>
-    <row r="61" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A61" s="1" t="s">
         <v>11</v>
       </c>
@@ -4721,7 +4701,7 @@
       </c>
       <c r="T61" s="1"/>
     </row>
-    <row r="62" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A62" s="1" t="s">
         <v>11</v>
       </c>
@@ -4773,7 +4753,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="63" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>11</v>
       </c>
@@ -4823,7 +4803,7 @@
       </c>
       <c r="T63" s="1"/>
     </row>
-    <row r="64" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A64" s="1" t="s">
         <v>11</v>
       </c>
@@ -4873,7 +4853,7 @@
       </c>
       <c r="T64" s="1"/>
     </row>
-    <row r="65" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A65" s="1" t="s">
         <v>11</v>
       </c>
@@ -4923,7 +4903,7 @@
       </c>
       <c r="T65" s="1"/>
     </row>
-    <row r="66" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A66" s="1" t="s">
         <v>11</v>
       </c>
@@ -4975,7 +4955,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="67" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A67" s="1" t="s">
         <v>11</v>
       </c>
@@ -5027,7 +5007,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="68" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A68" s="1" t="s">
         <v>11</v>
       </c>
@@ -5079,7 +5059,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="69" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A69" s="1" t="s">
         <v>11</v>
       </c>
@@ -5129,7 +5109,7 @@
       </c>
       <c r="T69" s="1"/>
     </row>
-    <row r="70" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A70" s="1" t="s">
         <v>11</v>
       </c>
@@ -5179,7 +5159,7 @@
       </c>
       <c r="T70" s="1"/>
     </row>
-    <row r="71" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A71" s="1" t="s">
         <v>11</v>
       </c>
@@ -5229,7 +5209,7 @@
       </c>
       <c r="T71" s="1"/>
     </row>
-    <row r="72" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A72" s="1" t="s">
         <v>11</v>
       </c>
@@ -5281,7 +5261,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="73" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A73" s="1" t="s">
         <v>11</v>
       </c>
@@ -5331,7 +5311,7 @@
       </c>
       <c r="T73" s="1"/>
     </row>
-    <row r="74" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A74" s="1" t="s">
         <v>11</v>
       </c>
@@ -5381,7 +5361,7 @@
       </c>
       <c r="T74" s="1"/>
     </row>
-    <row r="75" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A75" s="1" t="s">
         <v>11</v>
       </c>
@@ -5433,7 +5413,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="76" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A76" s="1" t="s">
         <v>11</v>
       </c>
@@ -5483,7 +5463,7 @@
       </c>
       <c r="T76" s="1"/>
     </row>
-    <row r="77" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A77" s="1" t="s">
         <v>11</v>
       </c>
@@ -5533,7 +5513,7 @@
       </c>
       <c r="T77" s="1"/>
     </row>
-    <row r="78" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A78" s="1" t="s">
         <v>11</v>
       </c>
@@ -5555,7 +5535,7 @@
         <v>194</v>
       </c>
       <c r="I78" s="1" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="J78" s="1">
         <v>10</v>
@@ -5585,7 +5565,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="79" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A79" s="1" t="s">
         <v>11</v>
       </c>
@@ -5609,7 +5589,9 @@
       <c r="I79" t="s">
         <v>155</v>
       </c>
-      <c r="J79" s="4"/>
+      <c r="J79" t="s">
+        <v>155</v>
+      </c>
       <c r="K79" s="4"/>
       <c r="L79" s="4"/>
       <c r="M79" s="4"/>
@@ -5633,7 +5615,7 @@
       </c>
       <c r="T79" s="4"/>
     </row>
-    <row r="80" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A80" s="1" t="s">
         <v>11</v>
       </c>
@@ -5655,9 +5637,11 @@
       <c r="G80" s="4"/>
       <c r="H80" s="4"/>
       <c r="I80" t="s">
-        <v>274</v>
-      </c>
-      <c r="J80" s="4"/>
+        <v>270</v>
+      </c>
+      <c r="J80" t="s">
+        <v>270</v>
+      </c>
       <c r="K80" s="4"/>
       <c r="L80" s="4"/>
       <c r="M80" s="4"/>
@@ -5681,7 +5665,7 @@
       </c>
       <c r="T80" s="4"/>
     </row>
-    <row r="81" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A81" s="1" t="s">
         <v>11</v>
       </c>
@@ -5705,7 +5689,9 @@
       <c r="I81" t="s">
         <v>252</v>
       </c>
-      <c r="J81" s="4"/>
+      <c r="J81" t="s">
+        <v>252</v>
+      </c>
       <c r="K81" s="4"/>
       <c r="L81" s="4"/>
       <c r="M81" s="4"/>
@@ -5729,7 +5715,7 @@
       </c>
       <c r="T81" s="4"/>
     </row>
-    <row r="82" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A82" s="1" t="s">
         <v>11</v>
       </c>
@@ -5753,7 +5739,9 @@
       <c r="I82" t="s">
         <v>253</v>
       </c>
-      <c r="J82" s="4"/>
+      <c r="J82" t="s">
+        <v>253</v>
+      </c>
       <c r="K82" s="4"/>
       <c r="L82" s="4"/>
       <c r="M82" s="4"/>
@@ -5777,7 +5765,7 @@
       </c>
       <c r="T82" s="4"/>
     </row>
-    <row r="83" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A83" s="1" t="s">
         <v>11</v>
       </c>
@@ -5799,9 +5787,11 @@
       <c r="G83" s="4"/>
       <c r="H83" s="4"/>
       <c r="I83" t="s">
-        <v>275</v>
-      </c>
-      <c r="J83" s="4"/>
+        <v>271</v>
+      </c>
+      <c r="J83" t="s">
+        <v>271</v>
+      </c>
       <c r="K83" s="4"/>
       <c r="L83" s="4"/>
       <c r="M83" s="4"/>
@@ -5825,7 +5815,7 @@
       </c>
       <c r="T83" s="4"/>
     </row>
-    <row r="84" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A84" s="1" t="s">
         <v>11</v>
       </c>
@@ -5849,7 +5839,9 @@
       <c r="I84" t="s">
         <v>155</v>
       </c>
-      <c r="J84" s="4"/>
+      <c r="J84" t="s">
+        <v>155</v>
+      </c>
       <c r="K84" s="4"/>
       <c r="L84" s="4"/>
       <c r="M84" s="4"/>
@@ -5873,7 +5865,7 @@
       </c>
       <c r="T84" s="4"/>
     </row>
-    <row r="85" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A85" s="1" t="s">
         <v>11</v>
       </c>
@@ -5897,7 +5889,9 @@
       <c r="I85" t="s">
         <v>252</v>
       </c>
-      <c r="J85" s="4"/>
+      <c r="J85" t="s">
+        <v>252</v>
+      </c>
       <c r="K85" s="4"/>
       <c r="L85" s="4"/>
       <c r="M85" s="4"/>
@@ -5921,7 +5915,7 @@
       </c>
       <c r="T85" s="4"/>
     </row>
-    <row r="86" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A86" s="1" t="s">
         <v>11</v>
       </c>
@@ -5943,9 +5937,11 @@
       <c r="G86" s="4"/>
       <c r="H86" s="4"/>
       <c r="I86" t="s">
-        <v>274</v>
-      </c>
-      <c r="J86" s="4"/>
+        <v>270</v>
+      </c>
+      <c r="J86" t="s">
+        <v>270</v>
+      </c>
       <c r="K86" s="4"/>
       <c r="L86" s="4"/>
       <c r="M86" s="4"/>
@@ -5969,7 +5965,7 @@
       </c>
       <c r="T86" s="4"/>
     </row>
-    <row r="87" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A87" s="1" t="s">
         <v>11</v>
       </c>
@@ -5993,7 +5989,9 @@
       <c r="I87" t="s">
         <v>155</v>
       </c>
-      <c r="J87" s="4"/>
+      <c r="J87" t="s">
+        <v>155</v>
+      </c>
       <c r="K87" s="4"/>
       <c r="L87" s="4"/>
       <c r="M87" s="4"/>
@@ -6017,7 +6015,7 @@
       </c>
       <c r="T87" s="4"/>
     </row>
-    <row r="88" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A88" s="1" t="s">
         <v>11</v>
       </c>
@@ -6041,7 +6039,9 @@
       <c r="I88" t="s">
         <v>155</v>
       </c>
-      <c r="J88" s="4"/>
+      <c r="J88" t="s">
+        <v>155</v>
+      </c>
       <c r="K88" s="4"/>
       <c r="L88" s="4"/>
       <c r="M88" s="4"/>
@@ -6065,7 +6065,7 @@
       </c>
       <c r="T88" s="4"/>
     </row>
-    <row r="89" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A89" s="1" t="s">
         <v>11</v>
       </c>
@@ -6089,7 +6089,9 @@
       <c r="I89" t="s">
         <v>252</v>
       </c>
-      <c r="J89" s="4"/>
+      <c r="J89" t="s">
+        <v>252</v>
+      </c>
       <c r="K89" s="4"/>
       <c r="L89" s="4"/>
       <c r="M89" s="4"/>
@@ -6113,7 +6115,7 @@
       </c>
       <c r="T89" s="4"/>
     </row>
-    <row r="90" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A90" s="1" t="s">
         <v>11</v>
       </c>
@@ -6137,7 +6139,9 @@
       <c r="I90" t="s">
         <v>252</v>
       </c>
-      <c r="J90" s="4"/>
+      <c r="J90" t="s">
+        <v>252</v>
+      </c>
       <c r="K90" s="4"/>
       <c r="L90" s="4"/>
       <c r="M90" s="4"/>
@@ -6161,7 +6165,7 @@
       </c>
       <c r="T90" s="4"/>
     </row>
-    <row r="91" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A91" s="1" t="s">
         <v>11</v>
       </c>
@@ -6185,7 +6189,9 @@
       <c r="I91" t="s">
         <v>252</v>
       </c>
-      <c r="J91" s="4"/>
+      <c r="J91" t="s">
+        <v>252</v>
+      </c>
       <c r="K91" s="4"/>
       <c r="L91" s="4"/>
       <c r="M91" s="4"/>
@@ -6209,7 +6215,7 @@
       </c>
       <c r="T91" s="4"/>
     </row>
-    <row r="92" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A92" s="1" t="s">
         <v>11</v>
       </c>
@@ -6233,7 +6239,9 @@
       <c r="I92" t="s">
         <v>253</v>
       </c>
-      <c r="J92" s="4"/>
+      <c r="J92" t="s">
+        <v>253</v>
+      </c>
       <c r="K92" s="4"/>
       <c r="L92" s="4"/>
       <c r="M92" s="4"/>
@@ -6257,7 +6265,7 @@
       </c>
       <c r="T92" s="4"/>
     </row>
-    <row r="93" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A93" s="1" t="s">
         <v>11</v>
       </c>
@@ -6279,9 +6287,11 @@
       <c r="G93" s="4"/>
       <c r="H93" s="4"/>
       <c r="I93" t="s">
-        <v>275</v>
-      </c>
-      <c r="J93" s="4"/>
+        <v>271</v>
+      </c>
+      <c r="J93" t="s">
+        <v>271</v>
+      </c>
       <c r="K93" s="4"/>
       <c r="L93" s="4"/>
       <c r="M93" s="4"/>
@@ -6305,7 +6315,7 @@
       </c>
       <c r="T93" s="4"/>
     </row>
-    <row r="94" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A94" s="1" t="s">
         <v>11</v>
       </c>
@@ -6329,7 +6339,9 @@
       <c r="I94" t="s">
         <v>253</v>
       </c>
-      <c r="J94" s="4"/>
+      <c r="J94" t="s">
+        <v>253</v>
+      </c>
       <c r="K94" s="4"/>
       <c r="L94" s="4"/>
       <c r="M94" s="4"/>
@@ -6353,7 +6365,7 @@
       </c>
       <c r="T94" s="4"/>
     </row>
-    <row r="95" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A95" s="1" t="s">
         <v>11</v>
       </c>
@@ -6377,7 +6389,9 @@
       <c r="I95" t="s">
         <v>253</v>
       </c>
-      <c r="J95" s="4"/>
+      <c r="J95" t="s">
+        <v>253</v>
+      </c>
       <c r="K95" s="4"/>
       <c r="L95" s="4"/>
       <c r="M95" s="4"/>
@@ -6401,7 +6415,7 @@
       </c>
       <c r="T95" s="4"/>
     </row>
-    <row r="96" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A96" s="1" t="s">
         <v>11</v>
       </c>
@@ -6423,9 +6437,11 @@
       <c r="G96" s="4"/>
       <c r="H96" s="4"/>
       <c r="I96" t="s">
-        <v>272</v>
-      </c>
-      <c r="J96" s="4"/>
+        <v>268</v>
+      </c>
+      <c r="J96" t="s">
+        <v>268</v>
+      </c>
       <c r="K96" s="4"/>
       <c r="L96" s="4"/>
       <c r="M96" s="4"/>
@@ -6449,7 +6465,7 @@
       </c>
       <c r="T96" s="4"/>
     </row>
-    <row r="97" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A97" s="1" t="s">
         <v>11</v>
       </c>
@@ -6473,7 +6489,9 @@
       <c r="I97" t="s">
         <v>155</v>
       </c>
-      <c r="J97" s="4"/>
+      <c r="J97" t="s">
+        <v>155</v>
+      </c>
       <c r="K97" s="4"/>
       <c r="L97" s="4"/>
       <c r="M97" s="4"/>
@@ -6497,7 +6515,7 @@
       </c>
       <c r="T97" s="4"/>
     </row>
-    <row r="98" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A98" s="1" t="s">
         <v>11</v>
       </c>
@@ -6521,7 +6539,9 @@
       <c r="I98" t="s">
         <v>252</v>
       </c>
-      <c r="J98" s="4"/>
+      <c r="J98" t="s">
+        <v>252</v>
+      </c>
       <c r="K98" s="4"/>
       <c r="L98" s="4"/>
       <c r="M98" s="4"/>
@@ -6545,7 +6565,7 @@
       </c>
       <c r="T98" s="4"/>
     </row>
-    <row r="99" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A99" s="1" t="s">
         <v>11</v>
       </c>
@@ -6567,9 +6587,11 @@
       <c r="G99" s="4"/>
       <c r="H99" s="4"/>
       <c r="I99" t="s">
-        <v>275</v>
-      </c>
-      <c r="J99" s="4"/>
+        <v>271</v>
+      </c>
+      <c r="J99" t="s">
+        <v>271</v>
+      </c>
       <c r="K99" s="4"/>
       <c r="L99" s="4"/>
       <c r="M99" s="4"/>
@@ -6593,7 +6615,7 @@
       </c>
       <c r="T99" s="4"/>
     </row>
-    <row r="100" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A100" s="1" t="s">
         <v>11</v>
       </c>
@@ -6617,7 +6639,9 @@
       <c r="I100" t="s">
         <v>155</v>
       </c>
-      <c r="J100" s="4"/>
+      <c r="J100" t="s">
+        <v>155</v>
+      </c>
       <c r="K100" s="4"/>
       <c r="L100" s="4"/>
       <c r="M100" s="4"/>
@@ -6641,7 +6665,7 @@
       </c>
       <c r="T100" s="4"/>
     </row>
-    <row r="101" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A101" s="1" t="s">
         <v>11</v>
       </c>
@@ -6665,7 +6689,9 @@
       <c r="I101" t="s">
         <v>253</v>
       </c>
-      <c r="J101" s="4"/>
+      <c r="J101" t="s">
+        <v>253</v>
+      </c>
       <c r="K101" s="4"/>
       <c r="L101" s="4"/>
       <c r="M101" s="4"/>
@@ -6689,7 +6715,7 @@
       </c>
       <c r="T101" s="4"/>
     </row>
-    <row r="102" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A102" s="1" t="s">
         <v>11</v>
       </c>
@@ -6713,7 +6739,9 @@
       <c r="I102" t="s">
         <v>253</v>
       </c>
-      <c r="J102" s="1"/>
+      <c r="J102" t="s">
+        <v>253</v>
+      </c>
       <c r="K102" s="1"/>
       <c r="L102" s="1"/>
       <c r="M102" s="1"/>
@@ -6737,7 +6765,7 @@
       </c>
       <c r="T102" s="1"/>
     </row>
-    <row r="103" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A103" s="1" t="s">
         <v>11</v>
       </c>
@@ -6758,16 +6786,19 @@
       </c>
       <c r="G103" s="4"/>
       <c r="H103" s="4"/>
-      <c r="I103" s="4" t="s">
-        <v>263</v>
-      </c>
-      <c r="J103" s="4"/>
+      <c r="I103" t="s">
+        <v>282</v>
+      </c>
+      <c r="J103">
+        <f>ROUNDUP((((SUM(TFO!T2:T18)/36)+(TFO!T19/36))*3),0)</f>
+        <v>133</v>
+      </c>
       <c r="K103" s="4"/>
       <c r="L103" s="4"/>
       <c r="M103" s="4"/>
       <c r="N103" s="4">
         <f>TFO!J23</f>
-        <v>62</v>
+        <v>0</v>
       </c>
       <c r="O103" s="4">
         <v>0</v>
@@ -6786,7 +6817,7 @@
       </c>
       <c r="T103" s="4"/>
     </row>
-    <row r="104" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A104" s="1" t="s">
         <v>11</v>
       </c>
@@ -6807,16 +6838,19 @@
       </c>
       <c r="G104" s="4"/>
       <c r="H104" s="4"/>
-      <c r="I104" s="4" t="s">
-        <v>264</v>
-      </c>
-      <c r="J104" s="4"/>
+      <c r="I104" t="s">
+        <v>283</v>
+      </c>
+      <c r="J104">
+        <f>ROUND(ROUNDUP(TFO!T19,0)/16,0)*2</f>
+        <v>40</v>
+      </c>
       <c r="K104" s="4"/>
       <c r="L104" s="4"/>
       <c r="M104" s="4"/>
       <c r="N104" s="4">
         <f>TFO!J24</f>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="O104" s="4">
         <v>0</v>
@@ -6835,7 +6869,7 @@
       </c>
       <c r="T104" s="4"/>
     </row>
-    <row r="105" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A105" s="1" t="s">
         <v>11</v>
       </c>
@@ -6856,16 +6890,19 @@
       </c>
       <c r="G105" s="4"/>
       <c r="H105" s="4"/>
-      <c r="I105" s="4" t="s">
-        <v>265</v>
-      </c>
-      <c r="J105" s="4"/>
+      <c r="I105" t="s">
+        <v>284</v>
+      </c>
+      <c r="J105">
+        <f>ROUND(+SUM(TFO!N2:N18)/6,0)*3</f>
+        <v>7944</v>
+      </c>
       <c r="K105" s="4"/>
       <c r="L105" s="4"/>
       <c r="M105" s="4"/>
       <c r="N105" s="4">
         <f>TFO!J25</f>
-        <v>33</v>
+        <v>0</v>
       </c>
       <c r="O105" s="4">
         <v>0</v>
@@ -6884,7 +6921,7 @@
       </c>
       <c r="T105" s="4"/>
     </row>
-    <row r="106" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A106" s="1" t="s">
         <v>11</v>
       </c>
@@ -6905,16 +6942,19 @@
       </c>
       <c r="G106" s="4"/>
       <c r="H106" s="4"/>
-      <c r="I106" s="4" t="s">
-        <v>266</v>
-      </c>
-      <c r="J106" s="4"/>
+      <c r="I106" t="s">
+        <v>285</v>
+      </c>
+      <c r="J106">
+        <f>ROUNDUP(+SUM(TFO!N2:N18)/4,0)*3</f>
+        <v>11916</v>
+      </c>
       <c r="K106" s="4"/>
       <c r="L106" s="4"/>
       <c r="M106" s="4"/>
       <c r="N106" s="4">
         <f>TFO!J26</f>
-        <v>51</v>
+        <v>0</v>
       </c>
       <c r="O106" s="4">
         <v>0</v>
@@ -6933,7 +6973,7 @@
       </c>
       <c r="T106" s="4"/>
     </row>
-    <row r="107" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A107" s="1" t="s">
         <v>11</v>
       </c>
@@ -6963,7 +7003,7 @@
       <c r="M107" s="4"/>
       <c r="N107" s="4">
         <f>TFO!J27</f>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O107" s="4">
         <v>0</v>
@@ -6982,7 +7022,7 @@
       </c>
       <c r="T107" s="4"/>
     </row>
-    <row r="108" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A108" s="1" t="s">
         <v>11</v>
       </c>
@@ -7012,7 +7052,7 @@
       <c r="M108" s="4"/>
       <c r="N108" s="4">
         <f>TFO!J28</f>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O108" s="4">
         <v>0</v>
@@ -7031,7 +7071,7 @@
       </c>
       <c r="T108" s="4"/>
     </row>
-    <row r="109" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A109" s="1" t="s">
         <v>11</v>
       </c>
@@ -7061,7 +7101,7 @@
       <c r="M109" s="4"/>
       <c r="N109" s="4">
         <f>TFO!J29</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O109" s="4">
         <v>0</v>
@@ -7080,7 +7120,7 @@
       </c>
       <c r="T109" s="4"/>
     </row>
-    <row r="110" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A110" s="1" t="s">
         <v>11</v>
       </c>
@@ -7110,7 +7150,7 @@
       <c r="M110" s="4"/>
       <c r="N110" s="4">
         <f>TFO!J30</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O110" s="4">
         <v>0</v>
@@ -7129,7 +7169,7 @@
       </c>
       <c r="T110" s="4"/>
     </row>
-    <row r="111" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A111" s="1" t="s">
         <v>11</v>
       </c>
@@ -7159,7 +7199,7 @@
       <c r="M111" s="4"/>
       <c r="N111" s="4">
         <f>TFO!J31</f>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O111" s="4">
         <v>0</v>
@@ -7178,7 +7218,7 @@
       </c>
       <c r="T111" s="4"/>
     </row>
-    <row r="112" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A112" s="1" t="s">
         <v>11</v>
       </c>
@@ -7206,7 +7246,7 @@
       <c r="M112" s="4"/>
       <c r="N112" s="4">
         <f>TFO!J32</f>
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="O112" s="4">
         <v>0</v>
@@ -7225,7 +7265,7 @@
       </c>
       <c r="T112" s="4"/>
     </row>
-    <row r="113" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A113" s="1" t="s">
         <v>11</v>
       </c>
@@ -7253,7 +7293,7 @@
       <c r="M113" s="4"/>
       <c r="N113" s="4">
         <f>TFO!J33</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O113" s="4">
         <v>1</v>
@@ -7272,7 +7312,7 @@
       </c>
       <c r="T113" s="4"/>
     </row>
-    <row r="114" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A114" s="1" t="s">
         <v>11</v>
       </c>
@@ -7300,7 +7340,7 @@
       <c r="M114" s="4"/>
       <c r="N114" s="4">
         <f>TFO!J34</f>
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="O114" s="4">
         <v>0</v>
@@ -7319,7 +7359,7 @@
       </c>
       <c r="T114" s="4"/>
     </row>
-    <row r="115" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A115" s="1" t="s">
         <v>11</v>
       </c>
@@ -7341,7 +7381,7 @@
       <c r="G115" s="4"/>
       <c r="H115" s="4"/>
       <c r="I115" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="J115" s="4"/>
       <c r="K115" s="4"/>
@@ -7368,7 +7408,7 @@
       </c>
       <c r="T115" s="4"/>
     </row>
-    <row r="116" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A116" s="1" t="s">
         <v>11</v>
       </c>
@@ -7398,7 +7438,7 @@
       <c r="M116" s="4"/>
       <c r="N116" s="4">
         <f>TFO!J36</f>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O116" s="4">
         <v>1</v>
@@ -7417,7 +7457,7 @@
       </c>
       <c r="T116" s="4"/>
     </row>
-    <row r="117" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A117" s="1" t="s">
         <v>11</v>
       </c>
@@ -7447,7 +7487,7 @@
       <c r="M117" s="4"/>
       <c r="N117" s="4">
         <f>TFO!J37</f>
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="O117" s="4">
         <v>0</v>
@@ -7476,37 +7516,37 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A6343EE0-D320-4977-9825-4200D3368BED}">
-  <dimension ref="A1:X37"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:X19"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.33203125" customWidth="1"/>
+    <col min="1" max="1" width="17.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.36328125" customWidth="1"/>
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.33203125" customWidth="1"/>
-    <col min="5" max="5" width="19.44140625" customWidth="1"/>
+    <col min="4" max="4" width="8.36328125" customWidth="1"/>
+    <col min="5" max="5" width="19.453125" customWidth="1"/>
     <col min="6" max="6" width="12" customWidth="1"/>
-    <col min="7" max="7" width="11.33203125" customWidth="1"/>
+    <col min="7" max="7" width="11.36328125" customWidth="1"/>
     <col min="8" max="8" width="38" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="46.6640625" customWidth="1"/>
-    <col min="10" max="10" width="43.33203125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="31.33203125" customWidth="1"/>
-    <col min="12" max="12" width="34.6640625" customWidth="1"/>
-    <col min="13" max="13" width="23.21875" customWidth="1"/>
-    <col min="14" max="14" width="34.88671875" customWidth="1"/>
-    <col min="15" max="15" width="26.77734375" customWidth="1"/>
-    <col min="16" max="16" width="39.33203125" customWidth="1"/>
-    <col min="17" max="17" width="13.77734375" customWidth="1"/>
-    <col min="18" max="18" width="33.44140625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="45.109375" customWidth="1"/>
-    <col min="20" max="20" width="40.44140625" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="49.88671875" customWidth="1"/>
-    <col min="22" max="22" width="25.109375" customWidth="1"/>
+    <col min="9" max="9" width="46.6328125" customWidth="1"/>
+    <col min="10" max="10" width="43.36328125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="31.36328125" customWidth="1"/>
+    <col min="12" max="12" width="34.6328125" customWidth="1"/>
+    <col min="13" max="13" width="23.1796875" customWidth="1"/>
+    <col min="14" max="14" width="34.90625" customWidth="1"/>
+    <col min="15" max="15" width="26.81640625" customWidth="1"/>
+    <col min="16" max="16" width="39.36328125" customWidth="1"/>
+    <col min="17" max="17" width="13.81640625" customWidth="1"/>
+    <col min="18" max="18" width="33.453125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="45.08984375" customWidth="1"/>
+    <col min="20" max="20" width="40.453125" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="49.90625" customWidth="1"/>
+    <col min="22" max="22" width="25.08984375" customWidth="1"/>
     <col min="23" max="23" width="17" customWidth="1"/>
-    <col min="24" max="24" width="15.5546875" customWidth="1"/>
+    <col min="24" max="24" width="15.54296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>196</v>
       </c>
@@ -7535,7 +7575,7 @@
         <v>204</v>
       </c>
       <c r="J1" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="K1" t="s">
         <v>205</v>
@@ -7544,7 +7584,7 @@
         <v>206</v>
       </c>
       <c r="M1" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="N1" t="s">
         <v>207</v>
@@ -7580,7 +7620,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>218</v>
       </c>
@@ -7610,7 +7650,7 @@
         <v>3.358291545501034</v>
       </c>
       <c r="J2" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="K2">
         <f>L2*30</f>
@@ -7620,7 +7660,7 @@
         <v>9386.496000000001</v>
       </c>
       <c r="M2" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="N2">
         <f t="shared" ref="N2:N18" si="0">L2/I2</f>
@@ -7640,7 +7680,7 @@
         <v>0.85</v>
       </c>
       <c r="S2" s="2" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="T2">
         <f t="shared" ref="T2:T19" si="1">Q2*R2*8*60*1.09/(C2*840*2.202)*3</f>
@@ -7654,14 +7694,14 @@
         <v>183.71918268499417</v>
       </c>
       <c r="W2" s="3" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="X2">
         <f>V2/72</f>
         <v>2.5516553150693633</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>218</v>
       </c>
@@ -7718,7 +7758,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>222</v>
       </c>
@@ -7783,7 +7823,7 @@
         <v>0.42808153681559535</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>224</v>
       </c>
@@ -7848,7 +7888,7 @@
         <v>2.7111830664987711</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>225</v>
       </c>
@@ -7913,7 +7953,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>226</v>
       </c>
@@ -7978,7 +8018,7 @@
         <v>0.18992832745236415</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>227</v>
       </c>
@@ -8043,7 +8083,7 @@
         <v>0.40861677010253639</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>228</v>
       </c>
@@ -8108,7 +8148,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>228</v>
       </c>
@@ -8173,7 +8213,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A11" t="s">
         <v>230</v>
       </c>
@@ -8238,7 +8278,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>231</v>
       </c>
@@ -8303,7 +8343,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A13" t="s">
         <v>232</v>
       </c>
@@ -8368,7 +8408,7 @@
         <v>0.70165756054775441</v>
       </c>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A14" t="s">
         <v>233</v>
       </c>
@@ -8433,7 +8473,7 @@
         <v>1.2948798803565318</v>
       </c>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A15" t="s">
         <v>234</v>
       </c>
@@ -8498,7 +8538,7 @@
         <v>0.77291166383862875</v>
       </c>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A16" t="s">
         <v>235</v>
       </c>
@@ -8563,7 +8603,7 @@
         <v>1.1040147594260059</v>
       </c>
     </row>
-    <row r="17" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A17" t="s">
         <v>236</v>
       </c>
@@ -8628,7 +8668,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A18" t="s">
         <v>237</v>
       </c>
@@ -8693,7 +8733,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:24" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:24" x14ac:dyDescent="0.35">
       <c r="A19" t="s">
         <v>238</v>
       </c>
@@ -8727,7 +8767,7 @@
         <v>2713.7828571428577</v>
       </c>
       <c r="M19" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="N19">
         <f>L19/I19</f>
@@ -8759,725 +8799,6 @@
       <c r="X19">
         <f t="shared" si="5"/>
         <v>0.118974377457405</v>
-      </c>
-    </row>
-    <row r="22" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
-        <v>0</v>
-      </c>
-      <c r="B22" t="s">
-        <v>1</v>
-      </c>
-      <c r="C22" t="s">
-        <v>254</v>
-      </c>
-      <c r="D22" t="s">
-        <v>2</v>
-      </c>
-      <c r="E22" t="s">
-        <v>285</v>
-      </c>
-      <c r="F22" t="s">
-        <v>3</v>
-      </c>
-      <c r="G22" t="s">
-        <v>4</v>
-      </c>
-      <c r="H22" t="s">
-        <v>44</v>
-      </c>
-      <c r="I22" t="s">
-        <v>45</v>
-      </c>
-      <c r="J22" t="s">
-        <v>270</v>
-      </c>
-      <c r="K22" t="s">
-        <v>269</v>
-      </c>
-      <c r="L22" t="s">
-        <v>5</v>
-      </c>
-      <c r="M22" t="s">
-        <v>6</v>
-      </c>
-      <c r="N22" t="s">
-        <v>7</v>
-      </c>
-      <c r="O22" t="s">
-        <v>8</v>
-      </c>
-      <c r="P22" t="s">
-        <v>9</v>
-      </c>
-      <c r="Q22" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="23" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
-        <v>11</v>
-      </c>
-      <c r="B23" t="s">
-        <v>12</v>
-      </c>
-      <c r="C23" t="s">
-        <v>123</v>
-      </c>
-      <c r="D23">
-        <v>1</v>
-      </c>
-      <c r="E23" t="s">
-        <v>124</v>
-      </c>
-      <c r="F23" t="s">
-        <v>125</v>
-      </c>
-      <c r="I23" t="s">
-        <v>263</v>
-      </c>
-      <c r="J23">
-        <v>62</v>
-      </c>
-      <c r="K23">
-        <f>J23</f>
-        <v>62</v>
-      </c>
-      <c r="L23">
-        <v>0</v>
-      </c>
-      <c r="M23">
-        <v>21</v>
-      </c>
-      <c r="N23">
-        <v>21</v>
-      </c>
-      <c r="O23">
-        <v>20</v>
-      </c>
-      <c r="P23">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
-        <v>11</v>
-      </c>
-      <c r="B24" t="s">
-        <v>12</v>
-      </c>
-      <c r="C24" t="s">
-        <v>123</v>
-      </c>
-      <c r="D24">
-        <v>2</v>
-      </c>
-      <c r="E24" t="s">
-        <v>126</v>
-      </c>
-      <c r="F24" t="s">
-        <v>125</v>
-      </c>
-      <c r="I24" t="s">
-        <v>264</v>
-      </c>
-      <c r="J24">
-        <v>2</v>
-      </c>
-      <c r="K24">
-        <f t="shared" ref="K24:K37" si="7">J24</f>
-        <v>2</v>
-      </c>
-      <c r="L24">
-        <v>0</v>
-      </c>
-      <c r="M24">
-        <v>1</v>
-      </c>
-      <c r="N24">
-        <v>1</v>
-      </c>
-      <c r="O24">
-        <v>0</v>
-      </c>
-      <c r="P24">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
-        <v>11</v>
-      </c>
-      <c r="B25" t="s">
-        <v>12</v>
-      </c>
-      <c r="C25" t="s">
-        <v>123</v>
-      </c>
-      <c r="D25">
-        <v>3</v>
-      </c>
-      <c r="E25" t="s">
-        <v>123</v>
-      </c>
-      <c r="F25" t="s">
-        <v>127</v>
-      </c>
-      <c r="I25" t="s">
-        <v>265</v>
-      </c>
-      <c r="J25">
-        <v>33</v>
-      </c>
-      <c r="K25">
-        <f t="shared" si="7"/>
-        <v>33</v>
-      </c>
-      <c r="L25">
-        <v>0</v>
-      </c>
-      <c r="M25">
-        <v>12</v>
-      </c>
-      <c r="N25">
-        <v>12</v>
-      </c>
-      <c r="O25">
-        <v>12</v>
-      </c>
-      <c r="P25">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
-        <v>11</v>
-      </c>
-      <c r="B26" t="s">
-        <v>12</v>
-      </c>
-      <c r="C26" t="s">
-        <v>123</v>
-      </c>
-      <c r="D26">
-        <v>4</v>
-      </c>
-      <c r="E26" t="s">
-        <v>123</v>
-      </c>
-      <c r="F26" t="s">
-        <v>128</v>
-      </c>
-      <c r="I26" t="s">
-        <v>266</v>
-      </c>
-      <c r="J26">
-        <v>51</v>
-      </c>
-      <c r="K26">
-        <f t="shared" si="7"/>
-        <v>51</v>
-      </c>
-      <c r="L26">
-        <v>0</v>
-      </c>
-      <c r="M26">
-        <v>17</v>
-      </c>
-      <c r="N26">
-        <v>17</v>
-      </c>
-      <c r="O26">
-        <v>17</v>
-      </c>
-      <c r="P26">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>11</v>
-      </c>
-      <c r="B27" t="s">
-        <v>12</v>
-      </c>
-      <c r="C27" t="s">
-        <v>123</v>
-      </c>
-      <c r="D27">
-        <v>5</v>
-      </c>
-      <c r="E27" t="s">
-        <v>129</v>
-      </c>
-      <c r="F27" t="s">
-        <v>127</v>
-      </c>
-      <c r="I27" t="s">
-        <v>147</v>
-      </c>
-      <c r="J27">
-        <v>6</v>
-      </c>
-      <c r="K27">
-        <f t="shared" si="7"/>
-        <v>6</v>
-      </c>
-      <c r="L27">
-        <v>0</v>
-      </c>
-      <c r="M27">
-        <v>2</v>
-      </c>
-      <c r="N27">
-        <v>2</v>
-      </c>
-      <c r="O27">
-        <v>2</v>
-      </c>
-      <c r="P27">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A28" t="s">
-        <v>11</v>
-      </c>
-      <c r="B28" t="s">
-        <v>12</v>
-      </c>
-      <c r="C28" t="s">
-        <v>123</v>
-      </c>
-      <c r="D28">
-        <v>6</v>
-      </c>
-      <c r="E28" t="s">
-        <v>130</v>
-      </c>
-      <c r="F28" t="s">
-        <v>127</v>
-      </c>
-      <c r="I28" t="s">
-        <v>147</v>
-      </c>
-      <c r="J28">
-        <v>6</v>
-      </c>
-      <c r="K28">
-        <f t="shared" si="7"/>
-        <v>6</v>
-      </c>
-      <c r="L28">
-        <v>0</v>
-      </c>
-      <c r="M28">
-        <v>2</v>
-      </c>
-      <c r="N28">
-        <v>2</v>
-      </c>
-      <c r="O28">
-        <v>2</v>
-      </c>
-      <c r="P28">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A29" t="s">
-        <v>11</v>
-      </c>
-      <c r="B29" t="s">
-        <v>12</v>
-      </c>
-      <c r="C29" t="s">
-        <v>123</v>
-      </c>
-      <c r="D29">
-        <v>7</v>
-      </c>
-      <c r="E29" t="s">
-        <v>29</v>
-      </c>
-      <c r="F29" t="s">
-        <v>29</v>
-      </c>
-      <c r="I29" t="s">
-        <v>155</v>
-      </c>
-      <c r="J29">
-        <v>3</v>
-      </c>
-      <c r="K29">
-        <f t="shared" si="7"/>
-        <v>3</v>
-      </c>
-      <c r="L29">
-        <v>0</v>
-      </c>
-      <c r="M29">
-        <v>1</v>
-      </c>
-      <c r="N29">
-        <v>1</v>
-      </c>
-      <c r="O29">
-        <v>1</v>
-      </c>
-      <c r="P29">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A30" t="s">
-        <v>11</v>
-      </c>
-      <c r="B30" t="s">
-        <v>12</v>
-      </c>
-      <c r="C30" t="s">
-        <v>123</v>
-      </c>
-      <c r="D30">
-        <v>8</v>
-      </c>
-      <c r="E30" t="s">
-        <v>131</v>
-      </c>
-      <c r="F30" t="s">
-        <v>106</v>
-      </c>
-      <c r="I30" t="s">
-        <v>155</v>
-      </c>
-      <c r="J30">
-        <v>3</v>
-      </c>
-      <c r="K30">
-        <f t="shared" si="7"/>
-        <v>3</v>
-      </c>
-      <c r="L30">
-        <v>0</v>
-      </c>
-      <c r="M30">
-        <v>1</v>
-      </c>
-      <c r="N30">
-        <v>1</v>
-      </c>
-      <c r="O30">
-        <v>1</v>
-      </c>
-      <c r="P30">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A31" t="s">
-        <v>11</v>
-      </c>
-      <c r="B31" t="s">
-        <v>12</v>
-      </c>
-      <c r="C31" t="s">
-        <v>123</v>
-      </c>
-      <c r="D31">
-        <v>9</v>
-      </c>
-      <c r="E31" t="s">
-        <v>132</v>
-      </c>
-      <c r="F31" t="s">
-        <v>133</v>
-      </c>
-      <c r="I31" t="s">
-        <v>147</v>
-      </c>
-      <c r="J31">
-        <v>6</v>
-      </c>
-      <c r="K31">
-        <f t="shared" si="7"/>
-        <v>6</v>
-      </c>
-      <c r="L31">
-        <v>0</v>
-      </c>
-      <c r="M31">
-        <v>2</v>
-      </c>
-      <c r="N31">
-        <v>2</v>
-      </c>
-      <c r="O31">
-        <v>2</v>
-      </c>
-      <c r="P31">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:24" x14ac:dyDescent="0.3">
-      <c r="A32" t="s">
-        <v>11</v>
-      </c>
-      <c r="B32" t="s">
-        <v>12</v>
-      </c>
-      <c r="C32" t="s">
-        <v>123</v>
-      </c>
-      <c r="D32">
-        <v>10</v>
-      </c>
-      <c r="E32" t="s">
-        <v>134</v>
-      </c>
-      <c r="I32" t="s">
-        <v>155</v>
-      </c>
-      <c r="J32">
-        <v>3</v>
-      </c>
-      <c r="K32">
-        <f t="shared" si="7"/>
-        <v>3</v>
-      </c>
-      <c r="L32">
-        <v>0</v>
-      </c>
-      <c r="M32">
-        <v>1</v>
-      </c>
-      <c r="N32">
-        <v>1</v>
-      </c>
-      <c r="O32">
-        <v>1</v>
-      </c>
-      <c r="P32">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A33" t="s">
-        <v>11</v>
-      </c>
-      <c r="B33" t="s">
-        <v>12</v>
-      </c>
-      <c r="C33" t="s">
-        <v>123</v>
-      </c>
-      <c r="D33">
-        <v>11</v>
-      </c>
-      <c r="E33" t="s">
-        <v>135</v>
-      </c>
-      <c r="I33" t="s">
-        <v>253</v>
-      </c>
-      <c r="J33">
-        <v>1</v>
-      </c>
-      <c r="K33">
-        <f t="shared" si="7"/>
-        <v>1</v>
-      </c>
-      <c r="L33">
-        <v>1</v>
-      </c>
-      <c r="M33">
-        <v>0</v>
-      </c>
-      <c r="N33">
-        <v>0</v>
-      </c>
-      <c r="O33">
-        <v>0</v>
-      </c>
-      <c r="P33">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A34" t="s">
-        <v>11</v>
-      </c>
-      <c r="B34" t="s">
-        <v>12</v>
-      </c>
-      <c r="C34" t="s">
-        <v>123</v>
-      </c>
-      <c r="D34">
-        <v>12</v>
-      </c>
-      <c r="E34" t="s">
-        <v>112</v>
-      </c>
-      <c r="I34" t="s">
-        <v>140</v>
-      </c>
-      <c r="J34">
-        <v>12</v>
-      </c>
-      <c r="K34">
-        <f t="shared" si="7"/>
-        <v>12</v>
-      </c>
-      <c r="L34">
-        <v>0</v>
-      </c>
-      <c r="M34">
-        <v>4</v>
-      </c>
-      <c r="N34">
-        <v>4</v>
-      </c>
-      <c r="O34">
-        <v>4</v>
-      </c>
-      <c r="P34">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A35" t="s">
-        <v>11</v>
-      </c>
-      <c r="B35" t="s">
-        <v>12</v>
-      </c>
-      <c r="C35" t="s">
-        <v>123</v>
-      </c>
-      <c r="D35">
-        <v>13</v>
-      </c>
-      <c r="E35" t="s">
-        <v>136</v>
-      </c>
-      <c r="F35" t="s">
-        <v>29</v>
-      </c>
-      <c r="I35" t="s">
-        <v>271</v>
-      </c>
-      <c r="J35">
-        <v>0</v>
-      </c>
-      <c r="K35">
-        <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="L35">
-        <v>0</v>
-      </c>
-      <c r="M35">
-        <v>0</v>
-      </c>
-      <c r="N35">
-        <v>0</v>
-      </c>
-      <c r="O35">
-        <v>0</v>
-      </c>
-      <c r="P35">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A36" t="s">
-        <v>11</v>
-      </c>
-      <c r="B36" t="s">
-        <v>12</v>
-      </c>
-      <c r="C36" t="s">
-        <v>123</v>
-      </c>
-      <c r="D36">
-        <v>15</v>
-      </c>
-      <c r="E36" t="s">
-        <v>157</v>
-      </c>
-      <c r="F36" t="s">
-        <v>157</v>
-      </c>
-      <c r="I36" t="s">
-        <v>253</v>
-      </c>
-      <c r="J36">
-        <v>1</v>
-      </c>
-      <c r="K36">
-        <f t="shared" si="7"/>
-        <v>1</v>
-      </c>
-      <c r="L36">
-        <v>1</v>
-      </c>
-      <c r="M36">
-        <v>0</v>
-      </c>
-      <c r="N36">
-        <v>0</v>
-      </c>
-      <c r="O36">
-        <v>0</v>
-      </c>
-      <c r="P36">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A37" t="s">
-        <v>11</v>
-      </c>
-      <c r="B37" t="s">
-        <v>12</v>
-      </c>
-      <c r="C37" t="s">
-        <v>123</v>
-      </c>
-      <c r="D37">
-        <v>16</v>
-      </c>
-      <c r="E37" t="s">
-        <v>31</v>
-      </c>
-      <c r="F37" t="s">
-        <v>42</v>
-      </c>
-      <c r="I37" t="s">
-        <v>147</v>
-      </c>
-      <c r="J37">
-        <v>6</v>
-      </c>
-      <c r="K37">
-        <f t="shared" si="7"/>
-        <v>6</v>
-      </c>
-      <c r="L37">
-        <v>0</v>
-      </c>
-      <c r="M37">
-        <v>2</v>
-      </c>
-      <c r="N37">
-        <v>2</v>
-      </c>
-      <c r="O37">
-        <v>2</v>
-      </c>
-      <c r="P37">
-        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>